<commit_message>
feat: enhance formatting functions and add tests for magnitude representation; update structure for December audit
</commit_message>
<xml_diff>
--- a/server/mpaStructure.xlsx
+++ b/server/mpaStructure.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:QT1"/>
+  <dimension ref="A1:QX1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -896,1845 +896,1865 @@
       </c>
       <c r="CP1" s="1" t="inlineStr">
         <is>
+          <t>PBT 2025-10-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2025-11-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2025-12-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
           <t>PBT Cost to Income Ratio</t>
         </is>
       </c>
-      <c r="CQ1" s="1" t="inlineStr">
+      <c r="CT1" s="1" t="inlineStr">
         <is>
           <t>PBT FULL YR % ACHVD</t>
         </is>
       </c>
-      <c r="CR1" s="1" t="inlineStr">
+      <c r="CU1" s="1" t="inlineStr">
         <is>
           <t>PBT 33 YTD % ACHVD</t>
         </is>
       </c>
-      <c r="CS1" s="1" t="inlineStr">
+      <c r="CV1" s="1" t="inlineStr">
         <is>
           <t>PBT Mthly Var</t>
         </is>
       </c>
-      <c r="CT1" s="1" t="inlineStr">
+      <c r="CW1" s="1" t="inlineStr">
         <is>
           <t>PBT 35 12-Month High</t>
         </is>
       </c>
-      <c r="CU1" s="1" t="inlineStr">
+      <c r="CX1" s="1" t="inlineStr">
         <is>
           <t>PBT 36 24-Month High</t>
         </is>
       </c>
-      <c r="CV1" s="1" t="inlineStr">
+      <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>PBT Exp Run Rate</t>
         </is>
       </c>
-      <c r="CW1" s="1" t="inlineStr">
+      <c r="CZ1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 100</t>
         </is>
       </c>
-      <c r="CX1" s="1" t="inlineStr">
+      <c r="DA1" s="1" t="inlineStr">
         <is>
           <t>PBT INT. INCOME &amp; OTHER LOAN-RELATED FEES 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="CY1" s="1" t="inlineStr">
+      <c r="DB1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00</t>
         </is>
       </c>
-      <c r="CZ1" s="1" t="inlineStr">
+      <c r="DC1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00</t>
         </is>
       </c>
-      <c r="DA1" s="1" t="inlineStr">
+      <c r="DD1" s="1" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="DB1" s="1" t="inlineStr">
+      <c r="DE1" s="1" t="inlineStr">
         <is>
           <t>PBT INTEREST EXPENSE 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="DC1" s="1" t="inlineStr">
+      <c r="DF1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="DD1" s="1" t="inlineStr">
+      <c r="DG1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="DE1" s="1" t="inlineStr">
+      <c r="DH1" s="1" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="DF1" s="1" t="inlineStr">
+      <c r="DI1" s="1" t="inlineStr">
         <is>
           <t>PBT INTERBRANCH 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="DG1" s="1" t="inlineStr">
+      <c r="DJ1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="DH1" s="1" t="inlineStr">
+      <c r="DK1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="DI1" s="1" t="inlineStr">
+      <c r="DL1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 104</t>
         </is>
       </c>
-      <c r="DJ1" s="1" t="inlineStr">
+      <c r="DM1" s="1" t="inlineStr">
         <is>
           <t>PBT SHARED INCOME 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="DK1" s="1" t="inlineStr">
+      <c r="DN1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="DL1" s="1" t="inlineStr">
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="DM1" s="1" t="inlineStr">
+      <c r="DP1" s="1" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="DN1" s="1" t="inlineStr">
+      <c r="DQ1" s="1" t="inlineStr">
         <is>
           <t>PBT ACCT MAINT. FEES 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="DO1" s="1" t="inlineStr">
+      <c r="DR1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="DP1" s="1" t="inlineStr">
+      <c r="DS1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="DQ1" s="1" t="inlineStr">
+      <c r="DT1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 108</t>
         </is>
       </c>
-      <c r="DR1" s="1" t="inlineStr">
+      <c r="DU1" s="1" t="inlineStr">
         <is>
           <t>PBT OTHER FEES &amp; COMMISSION 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="DS1" s="1" t="inlineStr">
+      <c r="DV1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-01 00:00:00__6</t>
         </is>
       </c>
-      <c r="DT1" s="1" t="inlineStr">
+      <c r="DW1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-01 00:00:00__6</t>
         </is>
       </c>
-      <c r="DU1" s="1" t="inlineStr">
+      <c r="DX1" s="1" t="inlineStr">
         <is>
           <t>92</t>
         </is>
       </c>
-      <c r="DV1" s="1" t="inlineStr">
+      <c r="DY1" s="1" t="inlineStr">
         <is>
           <t>PBT OPERATING EXPENSE 2025-06-29 00:00:00</t>
         </is>
       </c>
-      <c r="DW1" s="1" t="inlineStr">
+      <c r="DZ1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-07-29 00:00:00</t>
         </is>
       </c>
-      <c r="DX1" s="1" t="inlineStr">
+      <c r="EA1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025-08-29 00:00:00</t>
         </is>
       </c>
-      <c r="DY1" s="1" t="inlineStr">
+      <c r="EB1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 128</t>
         </is>
       </c>
-      <c r="DZ1" s="1" t="inlineStr">
+      <c r="EC1" s="1" t="inlineStr">
         <is>
           <t>DDA 2025 FULL YR BGT</t>
         </is>
       </c>
-      <c r="EA1" s="1" t="inlineStr">
+      <c r="ED1" s="1" t="inlineStr">
         <is>
           <t>DDA May-25</t>
         </is>
       </c>
-      <c r="EB1" s="1" t="inlineStr">
+      <c r="EE1" s="1" t="inlineStr">
         <is>
           <t>DDA Jun-25</t>
         </is>
       </c>
-      <c r="EC1" s="1" t="inlineStr">
+      <c r="EF1" s="1" t="inlineStr">
         <is>
           <t>DDA Jul-25</t>
         </is>
       </c>
-      <c r="ED1" s="1" t="inlineStr">
+      <c r="EG1" s="1" t="inlineStr">
         <is>
           <t>DDA MOM Variance</t>
         </is>
       </c>
-      <c r="EE1" s="1" t="inlineStr">
+      <c r="EH1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 134</t>
         </is>
       </c>
-      <c r="EF1" s="1" t="inlineStr">
+      <c r="EI1" s="1" t="inlineStr">
         <is>
           <t>DDA Dec-24</t>
         </is>
       </c>
-      <c r="EG1" s="1" t="inlineStr">
+      <c r="EJ1" s="1" t="inlineStr">
         <is>
           <t>DDA YTD Variance</t>
         </is>
       </c>
-      <c r="EH1" s="1" t="inlineStr">
+      <c r="EK1" s="1" t="inlineStr">
         <is>
           <t>DDA 112 12-Month High</t>
         </is>
       </c>
-      <c r="EI1" s="1" t="inlineStr">
+      <c r="EL1" s="1" t="inlineStr">
         <is>
           <t>DDA 24-Month High</t>
         </is>
       </c>
-      <c r="EJ1" s="1" t="inlineStr">
+      <c r="EM1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 139</t>
         </is>
       </c>
-      <c r="EK1" s="1" t="inlineStr">
+      <c r="EN1" s="1" t="inlineStr">
         <is>
           <t>SAV 2025 FULL YR BGT</t>
         </is>
       </c>
-      <c r="EL1" s="1" t="inlineStr">
+      <c r="EO1" s="1" t="inlineStr">
         <is>
           <t>SAV May-25</t>
         </is>
       </c>
-      <c r="EM1" s="1" t="inlineStr">
+      <c r="EP1" s="1" t="inlineStr">
         <is>
           <t>SAV Jun-25</t>
         </is>
       </c>
-      <c r="EN1" s="1" t="inlineStr">
+      <c r="EQ1" s="1" t="inlineStr">
         <is>
           <t>SAV Jul-25</t>
         </is>
       </c>
-      <c r="EO1" s="1" t="inlineStr">
+      <c r="ER1" s="1" t="inlineStr">
         <is>
           <t>SAV MOM Variance</t>
         </is>
       </c>
-      <c r="EP1" s="1" t="inlineStr">
+      <c r="ES1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 145</t>
         </is>
       </c>
-      <c r="EQ1" s="1" t="inlineStr">
+      <c r="ET1" s="1" t="inlineStr">
         <is>
           <t>SAV Dec-24</t>
         </is>
       </c>
-      <c r="ER1" s="1" t="inlineStr">
+      <c r="EU1" s="1" t="inlineStr">
         <is>
           <t>SAV YTD Variance</t>
         </is>
       </c>
-      <c r="ES1" s="1" t="inlineStr">
+      <c r="EV1" s="1" t="inlineStr">
         <is>
           <t>SAV 12-Month High</t>
         </is>
       </c>
-      <c r="ET1" s="1" t="inlineStr">
+      <c r="EW1" s="1" t="inlineStr">
         <is>
           <t>SAV 24-Month High__2</t>
         </is>
       </c>
-      <c r="EU1" s="1" t="inlineStr">
+      <c r="EX1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 150</t>
         </is>
       </c>
-      <c r="EV1" s="1" t="inlineStr">
+      <c r="EY1" s="1" t="inlineStr">
         <is>
           <t>DP DOMICILIARY DEPOSITS 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="EW1" s="1" t="inlineStr">
+      <c r="EZ1" s="1" t="inlineStr">
         <is>
           <t>DP 2025-07-01 00:00:00__8</t>
         </is>
       </c>
-      <c r="EX1" s="1" t="inlineStr">
+      <c r="FA1" s="1" t="inlineStr">
         <is>
           <t>DP May-25</t>
         </is>
       </c>
-      <c r="EY1" s="1" t="inlineStr">
+      <c r="FB1" s="1" t="inlineStr">
         <is>
           <t>DP MOM VARIANCE</t>
         </is>
       </c>
-      <c r="EZ1" s="1" t="inlineStr">
+      <c r="FC1" s="1" t="inlineStr">
         <is>
           <t>unnamed__9</t>
         </is>
       </c>
-      <c r="FA1" s="1" t="inlineStr">
+      <c r="FD1" s="1" t="inlineStr">
         <is>
           <t>DP 2024-12-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="FB1" s="1" t="inlineStr">
+      <c r="FE1" s="1" t="inlineStr">
         <is>
           <t>DP YTD Variance</t>
         </is>
       </c>
-      <c r="FC1" s="1" t="inlineStr">
+      <c r="FF1" s="1" t="inlineStr">
         <is>
           <t>DP 137 12-Month High</t>
         </is>
       </c>
-      <c r="FD1" s="1" t="inlineStr">
+      <c r="FG1" s="1" t="inlineStr">
         <is>
           <t>DP 24-Month High__3</t>
         </is>
       </c>
-      <c r="FE1" s="1" t="inlineStr">
+      <c r="FH1" s="1" t="inlineStr">
         <is>
           <t>unnamed__10</t>
         </is>
       </c>
-      <c r="FF1" s="1" t="inlineStr">
+      <c r="FI1" s="1" t="inlineStr">
         <is>
           <t>FD 2025 FULL YR BGT</t>
         </is>
       </c>
-      <c r="FG1" s="1" t="inlineStr">
+      <c r="FJ1" s="1" t="inlineStr">
         <is>
           <t>FD May-25</t>
         </is>
       </c>
-      <c r="FH1" s="1" t="inlineStr">
+      <c r="FK1" s="1" t="inlineStr">
         <is>
           <t>FD Jun-25</t>
         </is>
       </c>
-      <c r="FI1" s="1" t="inlineStr">
+      <c r="FL1" s="1" t="inlineStr">
         <is>
           <t>FD Jul-25</t>
         </is>
       </c>
-      <c r="FJ1" s="1" t="inlineStr">
+      <c r="FM1" s="1" t="inlineStr">
         <is>
           <t>FD MOM Variance</t>
         </is>
       </c>
-      <c r="FK1" s="1" t="inlineStr">
+      <c r="FN1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 166</t>
         </is>
       </c>
-      <c r="FL1" s="1" t="inlineStr">
+      <c r="FO1" s="1" t="inlineStr">
         <is>
           <t>FD Dec-24</t>
         </is>
       </c>
-      <c r="FM1" s="1" t="inlineStr">
+      <c r="FP1" s="1" t="inlineStr">
         <is>
           <t>FD YTD Variance</t>
         </is>
       </c>
-      <c r="FN1" s="1" t="inlineStr">
+      <c r="FQ1" s="1" t="inlineStr">
         <is>
           <t>FD 150 12-Month High</t>
         </is>
       </c>
-      <c r="FO1" s="1" t="inlineStr">
+      <c r="FR1" s="1" t="inlineStr">
         <is>
           <t>FD 151 24-Month High</t>
         </is>
       </c>
-      <c r="FP1" s="1" t="inlineStr">
+      <c r="FS1" s="1" t="inlineStr">
         <is>
           <t>FD Jul-25__2</t>
         </is>
       </c>
-      <c r="FQ1" s="1" t="inlineStr">
+      <c r="FT1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 172</t>
         </is>
       </c>
-      <c r="FR1" s="1" t="inlineStr">
+      <c r="FU1" s="1" t="inlineStr">
         <is>
           <t>DP TOTAL DEPOSITS 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="FS1" s="1" t="inlineStr">
+      <c r="FV1" s="1" t="inlineStr">
         <is>
           <t>DP 2025-07-01 00:00:00__10</t>
         </is>
       </c>
-      <c r="FT1" s="1" t="inlineStr">
+      <c r="FW1" s="1" t="inlineStr">
         <is>
           <t>DP Jun-25</t>
         </is>
       </c>
-      <c r="FU1" s="1" t="inlineStr">
+      <c r="FX1" s="1" t="inlineStr">
         <is>
           <t>DP MOM Variance</t>
         </is>
       </c>
-      <c r="FV1" s="1" t="inlineStr">
+      <c r="FY1" s="1" t="inlineStr">
         <is>
           <t>unnamed__13</t>
         </is>
       </c>
-      <c r="FW1" s="1" t="inlineStr">
+      <c r="FZ1" s="1" t="inlineStr">
         <is>
           <t>DP 2024-12-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="FX1" s="1" t="inlineStr">
+      <c r="GA1" s="1" t="inlineStr">
         <is>
           <t>DP 162 YTD Variance</t>
         </is>
       </c>
-      <c r="FY1" s="1" t="inlineStr">
+      <c r="GB1" s="1" t="inlineStr">
         <is>
           <t>DP 12-Month High__2</t>
         </is>
       </c>
-      <c r="FZ1" s="1" t="inlineStr">
+      <c r="GC1" s="1" t="inlineStr">
         <is>
           <t>DP 363.1055172413794 24-Month High</t>
         </is>
       </c>
-      <c r="GA1" s="1" t="inlineStr">
+      <c r="GD1" s="1" t="inlineStr">
         <is>
           <t>362.719</t>
         </is>
       </c>
-      <c r="GB1" s="1" t="inlineStr">
+      <c r="GE1" s="1" t="inlineStr">
         <is>
           <t>DP 2025 FULL YR BGT</t>
         </is>
       </c>
-      <c r="GC1" s="1" t="inlineStr">
+      <c r="GF1" s="1" t="inlineStr">
         <is>
           <t>DP May-25__2</t>
         </is>
       </c>
-      <c r="GD1" s="1" t="inlineStr">
+      <c r="GG1" s="1" t="inlineStr">
         <is>
           <t>DP Jun-25__2</t>
         </is>
       </c>
-      <c r="GE1" s="1" t="inlineStr">
+      <c r="GH1" s="1" t="inlineStr">
         <is>
           <t>DP Jul-25</t>
         </is>
       </c>
-      <c r="GF1" s="1" t="inlineStr">
+      <c r="GI1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 187</t>
         </is>
       </c>
-      <c r="GG1" s="1" t="inlineStr">
+      <c r="GJ1" s="1" t="inlineStr">
         <is>
           <t>DP Dec-24</t>
         </is>
       </c>
-      <c r="GH1" s="1" t="inlineStr">
+      <c r="GK1" s="1" t="inlineStr">
         <is>
           <t>DP YTD Variance__2</t>
         </is>
       </c>
-      <c r="GI1" s="1" t="inlineStr">
+      <c r="GL1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 190</t>
         </is>
       </c>
-      <c r="GJ1" s="1" t="inlineStr">
+      <c r="GM1" s="1" t="inlineStr">
         <is>
           <t>TRA 1589 RISK ASSETS ($) FCY 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="GK1" s="1" t="inlineStr">
-        <is>
-          <t>TRA 1535.35 RISK ASSETS ($) FCY 2025-08-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="GL1" s="1" t="inlineStr">
-        <is>
-          <t>TRA 1479.44 RISK ASSETS ($) FCY 2025-09-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="GM1" s="1" t="inlineStr">
+      <c r="GN1" s="1" t="inlineStr">
+        <is>
+          <t>TRA 1535.35 2025-07-01 00:00:00__2</t>
+        </is>
+      </c>
+      <c r="GO1" s="1" t="inlineStr">
+        <is>
+          <t>TRA 1535.13 2025-08-01 00:00:00__2</t>
+        </is>
+      </c>
+      <c r="GP1" s="1" t="inlineStr">
         <is>
           <t>unnamed__16</t>
         </is>
       </c>
-      <c r="GN1" s="1" t="inlineStr">
+      <c r="GQ1" s="1" t="inlineStr">
         <is>
           <t>TRA 2024-12-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="GO1" s="1" t="inlineStr">
+      <c r="GR1" s="1" t="inlineStr">
         <is>
           <t>TRA MOM Variance__2</t>
         </is>
       </c>
-      <c r="GP1" s="1" t="inlineStr">
+      <c r="GS1" s="1" t="inlineStr">
         <is>
           <t>TRA YTD Variance</t>
         </is>
       </c>
-      <c r="GQ1" s="1" t="inlineStr">
+      <c r="GT1" s="1" t="inlineStr">
         <is>
           <t>179</t>
         </is>
       </c>
-      <c r="GR1" s="1" t="inlineStr">
+      <c r="GU1" s="1" t="inlineStr">
         <is>
           <t>TRA TOTAL RISK ASSETS 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="GS1" s="1" t="inlineStr">
+      <c r="GV1" s="1" t="inlineStr">
         <is>
           <t>TRA 2025-07-01 00:00:00__11</t>
         </is>
       </c>
-      <c r="GT1" s="1" t="inlineStr">
+      <c r="GW1" s="1" t="inlineStr">
         <is>
           <t>TRA 2025-08-01 00:00:00__11</t>
         </is>
       </c>
-      <c r="GU1" s="1" t="inlineStr">
+      <c r="GX1" s="1" t="inlineStr">
         <is>
           <t>unnamed__17</t>
         </is>
       </c>
-      <c r="GV1" s="1" t="inlineStr">
+      <c r="GY1" s="1" t="inlineStr">
         <is>
           <t>TRA 2024-12-01 00:00:00__6</t>
         </is>
       </c>
-      <c r="GW1" s="1" t="inlineStr">
+      <c r="GZ1" s="1" t="inlineStr">
         <is>
           <t>TRA YTD Variance__2</t>
         </is>
       </c>
-      <c r="GX1" s="1" t="inlineStr">
+      <c r="HA1" s="1" t="inlineStr">
         <is>
           <t>TRA Loan to Dep</t>
         </is>
       </c>
-      <c r="GY1" s="1" t="inlineStr">
+      <c r="HB1" s="1" t="inlineStr">
         <is>
           <t>unnamed__18</t>
         </is>
       </c>
-      <c r="GZ1" s="1" t="inlineStr">
+      <c r="HC1" s="1" t="inlineStr">
         <is>
           <t>TRA 187 RETAIL LOANS 2025 FULL YR BGT</t>
         </is>
       </c>
-      <c r="HA1" s="1" t="inlineStr">
+      <c r="HD1" s="1" t="inlineStr">
         <is>
           <t>TRA 2025-06-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="HB1" s="1" t="inlineStr">
+      <c r="HE1" s="1" t="inlineStr">
         <is>
           <t>TRA 2025-07-01 00:00:00__12</t>
         </is>
       </c>
-      <c r="HC1" s="1" t="inlineStr">
+      <c r="HF1" s="1" t="inlineStr">
         <is>
           <t>TRA May-25</t>
         </is>
       </c>
-      <c r="HD1" s="1" t="inlineStr">
+      <c r="HG1" s="1" t="inlineStr">
         <is>
           <t>unnamed__19</t>
         </is>
       </c>
-      <c r="HE1" s="1" t="inlineStr">
+      <c r="HH1" s="1" t="inlineStr">
         <is>
           <t>TRA 2024-12-01 00:00:00__7</t>
         </is>
       </c>
-      <c r="HF1" s="1" t="inlineStr">
+      <c r="HI1" s="1" t="inlineStr">
         <is>
           <t>TRA 195 YTD Variance</t>
         </is>
       </c>
-      <c r="HG1" s="1" t="inlineStr">
+      <c r="HJ1" s="1" t="inlineStr">
         <is>
           <t>205</t>
         </is>
       </c>
-      <c r="HH1" s="1" t="inlineStr">
-        <is>
-          <t>unnamed__20</t>
-        </is>
-      </c>
-      <c r="HI1" s="1" t="inlineStr">
-        <is>
-          <t>TRA BONDS AND GUARANTEES VOLUME 2025 FULL YR BGT</t>
-        </is>
-      </c>
-      <c r="HJ1" s="1" t="inlineStr">
-        <is>
-          <t>TRA 2025-06-01 00:00:00__4</t>
-        </is>
-      </c>
       <c r="HK1" s="1" t="inlineStr">
         <is>
-          <t>TRA 2025-07-01 00:00:00__13</t>
+          <t>TRA BONDS AND GUARANTEES 2025 FULL YR BGT</t>
         </is>
       </c>
       <c r="HL1" s="1" t="inlineStr">
         <is>
+          <t>TRA VOLUME 2025-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="HM1" s="1" t="inlineStr">
+        <is>
+          <t>TRA 2025-11-01 00:00:00__13</t>
+        </is>
+      </c>
+      <c r="HN1" s="1" t="inlineStr">
+        <is>
           <t>TRA Jun-25</t>
         </is>
       </c>
-      <c r="HM1" s="1" t="inlineStr">
+      <c r="HO1" s="1" t="inlineStr">
         <is>
           <t>214</t>
         </is>
       </c>
-      <c r="HN1" s="1" t="inlineStr">
+      <c r="HP1" s="1" t="inlineStr">
+        <is>
+          <t>TRA 2020-01-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="HQ1" s="1" t="inlineStr">
         <is>
           <t>TRA B&amp;G Fees 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="HO1" s="1" t="inlineStr">
+      <c r="HR1" s="1" t="inlineStr">
+        <is>
+          <t>TRA 2025-10-01 00:00:00__4</t>
+        </is>
+      </c>
+      <c r="HS1" s="1" t="inlineStr">
         <is>
           <t>TRA 2025-07-01 00:00:00__14</t>
         </is>
       </c>
-      <c r="HP1" s="1" t="inlineStr">
+      <c r="HT1" s="1" t="inlineStr">
         <is>
           <t>TRA Jul-25</t>
         </is>
       </c>
-      <c r="HQ1" s="1" t="inlineStr">
+      <c r="HU1" s="1" t="inlineStr">
         <is>
           <t>unnamed__21</t>
         </is>
       </c>
-      <c r="HR1" s="1" t="inlineStr">
+      <c r="HV1" s="1" t="inlineStr">
         <is>
           <t>AB 224 AGENCY BANKING PERFORMANCE No of Transaction 2025-07-01 00:00:00</t>
         </is>
       </c>
-      <c r="HS1" s="1" t="inlineStr">
+      <c r="HW1" s="1" t="inlineStr">
         <is>
           <t>AB Jul-25</t>
         </is>
       </c>
-      <c r="HT1" s="1" t="inlineStr">
+      <c r="HX1" s="1" t="inlineStr">
         <is>
           <t>AB VAR</t>
         </is>
       </c>
-      <c r="HU1" s="1" t="inlineStr">
+      <c r="HY1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 232</t>
         </is>
       </c>
-      <c r="HV1" s="1" t="inlineStr">
+      <c r="HZ1" s="1" t="inlineStr">
         <is>
           <t>AB VALUE 2025-09-01 00:00:00</t>
         </is>
       </c>
-      <c r="HW1" s="1" t="inlineStr">
+      <c r="IA1" s="1" t="inlineStr">
         <is>
           <t>AB `` 2025-07-01 00:00:00</t>
         </is>
       </c>
-      <c r="HX1" s="1" t="inlineStr">
+      <c r="IB1" s="1" t="inlineStr">
         <is>
           <t>AB 1000 VAR</t>
         </is>
       </c>
-      <c r="HY1" s="1" t="inlineStr">
+      <c r="IC1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 236</t>
         </is>
       </c>
-      <c r="HZ1" s="1" t="inlineStr">
+      <c r="ID1" s="1" t="inlineStr">
         <is>
           <t>AB INCOME 2025-07-01 00:00:00</t>
         </is>
       </c>
-      <c r="IA1" s="1" t="inlineStr">
+      <c r="IE1" s="1" t="inlineStr">
         <is>
           <t>AB Jun-25</t>
         </is>
       </c>
-      <c r="IB1" s="1" t="inlineStr">
+      <c r="IF1" s="1" t="inlineStr">
         <is>
           <t>AB VAR__2</t>
         </is>
       </c>
-      <c r="IC1" s="1" t="inlineStr">
+      <c r="IG1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 240</t>
         </is>
       </c>
-      <c r="ID1" s="1" t="inlineStr">
+      <c r="IH1" s="1" t="inlineStr">
         <is>
           <t>AB Electronic Fees income 2025-06-01 00:00:00</t>
         </is>
       </c>
-      <c r="IE1" s="1" t="inlineStr">
+      <c r="II1" s="1" t="inlineStr">
         <is>
           <t>AB 2025-07-01 00:00:00__15</t>
         </is>
       </c>
-      <c r="IF1" s="1" t="inlineStr">
+      <c r="IJ1" s="1" t="inlineStr">
         <is>
           <t>AB Jul-25__2</t>
         </is>
       </c>
-      <c r="IG1" s="1" t="inlineStr">
+      <c r="IK1" s="1" t="inlineStr">
         <is>
           <t>218</t>
         </is>
       </c>
-      <c r="IH1" s="1" t="inlineStr">
+      <c r="IL1" s="1" t="inlineStr">
         <is>
           <t>AO C/A Opened - Total</t>
         </is>
       </c>
-      <c r="II1" s="1" t="inlineStr">
+      <c r="IM1" s="1" t="inlineStr">
         <is>
           <t>AO C/A Opened - Funded</t>
         </is>
       </c>
-      <c r="IJ1" s="1" t="inlineStr">
+      <c r="IN1" s="1" t="inlineStr">
         <is>
           <t>AO C/A Opened - Unfunded</t>
         </is>
       </c>
-      <c r="IK1" s="1" t="inlineStr">
+      <c r="IO1" s="1" t="inlineStr">
         <is>
           <t>AO S/A Opened - Total</t>
         </is>
       </c>
-      <c r="IL1" s="1" t="inlineStr">
+      <c r="IP1" s="1" t="inlineStr">
         <is>
           <t>AO S/A Opened - Funded</t>
         </is>
       </c>
-      <c r="IM1" s="1" t="inlineStr">
+      <c r="IQ1" s="1" t="inlineStr">
         <is>
           <t>AO S/A Opened - Unfunded</t>
         </is>
       </c>
-      <c r="IN1" s="1" t="inlineStr">
+      <c r="IR1" s="1" t="inlineStr">
         <is>
           <t>AO Total Accounts opened</t>
         </is>
       </c>
-      <c r="IO1" s="1" t="inlineStr">
+      <c r="IS1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 248</t>
         </is>
       </c>
-      <c r="IP1" s="1" t="inlineStr">
-        <is>
-          <t>CDS1 No. of Cards Issued</t>
-        </is>
-      </c>
-      <c r="IQ1" s="1" t="inlineStr">
-        <is>
-          <t>CDS1 ACTIVE</t>
-        </is>
-      </c>
-      <c r="IR1" s="1" t="inlineStr">
-        <is>
-          <t>CDS1 INACTIVE</t>
-        </is>
-      </c>
-      <c r="IS1" s="1" t="inlineStr">
+      <c r="IT1" s="1" t="inlineStr">
+        <is>
+          <t>AO 224 CARDS NOVEMBER No. of Cards Issued</t>
+        </is>
+      </c>
+      <c r="IU1" s="1" t="inlineStr">
+        <is>
+          <t>AO 234 ACTIVE</t>
+        </is>
+      </c>
+      <c r="IV1" s="1" t="inlineStr">
+        <is>
+          <t>AO 235 INACTIVE</t>
+        </is>
+      </c>
+      <c r="IW1" s="1" t="inlineStr">
         <is>
           <t>223</t>
         </is>
       </c>
-      <c r="IT1" s="1" t="inlineStr">
-        <is>
-          <t>CDS2 No. of Cards Issued</t>
-        </is>
-      </c>
-      <c r="IU1" s="1" t="inlineStr">
-        <is>
-          <t>CDS2 ACTIVE</t>
-        </is>
-      </c>
-      <c r="IV1" s="1" t="inlineStr">
-        <is>
-          <t>CDS2 INACTIVE</t>
-        </is>
-      </c>
-      <c r="IW1" s="1" t="inlineStr">
-        <is>
-          <t>223__2</t>
-        </is>
-      </c>
       <c r="IX1" s="1" t="inlineStr">
         <is>
+          <t>AO 224 CARDS DECEMBER No. of Cards Issued</t>
+        </is>
+      </c>
+      <c r="IY1" s="1" t="inlineStr">
+        <is>
+          <t>AO 234 ACTIVE__2</t>
+        </is>
+      </c>
+      <c r="IZ1" s="1" t="inlineStr">
+        <is>
+          <t>AO 235 INACTIVE__2</t>
+        </is>
+      </c>
+      <c r="JA1" s="1" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="JB1" s="1" t="inlineStr">
+        <is>
           <t>CE May-25</t>
         </is>
       </c>
-      <c r="IY1" s="1" t="inlineStr">
+      <c r="JC1" s="1" t="inlineStr">
         <is>
           <t>CE Jun-25</t>
         </is>
       </c>
-      <c r="IZ1" s="1" t="inlineStr">
+      <c r="JD1" s="1" t="inlineStr">
         <is>
           <t>CE Jul-25</t>
         </is>
       </c>
-      <c r="JA1" s="1" t="inlineStr">
+      <c r="JE1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 260</t>
         </is>
       </c>
-      <c r="JB1" s="1" t="inlineStr">
+      <c r="JF1" s="1" t="inlineStr">
         <is>
           <t>AOB May-25</t>
         </is>
       </c>
-      <c r="JC1" s="1" t="inlineStr">
+      <c r="JG1" s="1" t="inlineStr">
         <is>
           <t>AOB Jun-25</t>
         </is>
       </c>
-      <c r="JD1" s="1" t="inlineStr">
+      <c r="JH1" s="1" t="inlineStr">
         <is>
           <t>AOB Jul-25</t>
         </is>
       </c>
-      <c r="JE1" s="1" t="inlineStr">
+      <c r="JI1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 264</t>
         </is>
       </c>
-      <c r="JF1" s="1" t="inlineStr">
+      <c r="JJ1" s="1" t="inlineStr">
         <is>
           <t>AOB OTHERS Dormant Accounts 2020-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="JG1" s="1" t="inlineStr">
+      <c r="JK1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-02-01 00:00:00</t>
         </is>
       </c>
-      <c r="JH1" s="1" t="inlineStr">
+      <c r="JL1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-03-01 00:00:00</t>
         </is>
       </c>
-      <c r="JI1" s="1" t="inlineStr">
+      <c r="JM1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-04-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JJ1" s="1" t="inlineStr">
+      <c r="JN1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-05-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JK1" s="1" t="inlineStr">
+      <c r="JO1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-06-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JL1" s="1" t="inlineStr">
+      <c r="JP1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-07-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JM1" s="1" t="inlineStr">
+      <c r="JQ1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-08-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JN1" s="1" t="inlineStr">
+      <c r="JR1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-09-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JO1" s="1" t="inlineStr">
+      <c r="JS1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-10-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JP1" s="1" t="inlineStr">
+      <c r="JT1" s="1" t="inlineStr">
         <is>
           <t>AOB 2020-11-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JQ1" s="1" t="inlineStr">
+      <c r="JU1" s="1" t="inlineStr">
         <is>
           <t>AOB 230 2020-12-01 00:00:00</t>
         </is>
       </c>
-      <c r="JR1" s="1" t="inlineStr">
+      <c r="JV1" s="1" t="inlineStr">
         <is>
           <t>AOB OTHERS Dormant Accounts 2021-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="JS1" s="1" t="inlineStr">
+      <c r="JW1" s="1" t="inlineStr">
         <is>
           <t>AOB 231 2021-02-01 00:00:00</t>
         </is>
       </c>
-      <c r="JT1" s="1" t="inlineStr">
+      <c r="JX1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-03-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JU1" s="1" t="inlineStr">
+      <c r="JY1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-04-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JV1" s="1" t="inlineStr">
+      <c r="JZ1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-05-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JW1" s="1" t="inlineStr">
+      <c r="KA1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-06-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JX1" s="1" t="inlineStr">
+      <c r="KB1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-07-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JY1" s="1" t="inlineStr">
+      <c r="KC1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-08-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="JZ1" s="1" t="inlineStr">
+      <c r="KD1" s="1" t="inlineStr">
         <is>
           <t>AOB 232 2021-09-01 00:00:00</t>
         </is>
       </c>
-      <c r="KA1" s="1" t="inlineStr">
+      <c r="KE1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-10-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KB1" s="1" t="inlineStr">
+      <c r="KF1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-11-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KC1" s="1" t="inlineStr">
+      <c r="KG1" s="1" t="inlineStr">
         <is>
           <t>AOB 2021-12-01 00:00:00</t>
         </is>
       </c>
-      <c r="KD1" s="1" t="inlineStr">
+      <c r="KH1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-01-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KE1" s="1" t="inlineStr">
+      <c r="KI1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-02-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KF1" s="1" t="inlineStr">
+      <c r="KJ1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-03-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KG1" s="1" t="inlineStr">
+      <c r="KK1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-04-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KH1" s="1" t="inlineStr">
+      <c r="KL1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-05-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KI1" s="1" t="inlineStr">
+      <c r="KM1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-06-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KJ1" s="1" t="inlineStr">
+      <c r="KN1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-07-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KK1" s="1" t="inlineStr">
+      <c r="KO1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-08-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KL1" s="1" t="inlineStr">
+      <c r="KP1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-09-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KM1" s="1" t="inlineStr">
+      <c r="KQ1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-10-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KN1" s="1" t="inlineStr">
+      <c r="KR1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-11-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KO1" s="1" t="inlineStr">
+      <c r="KS1" s="1" t="inlineStr">
         <is>
           <t>AOB 2022-12-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KP1" s="1" t="inlineStr">
+      <c r="KT1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-01-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KQ1" s="1" t="inlineStr">
+      <c r="KU1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-02-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KR1" s="1" t="inlineStr">
+      <c r="KV1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-03-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KS1" s="1" t="inlineStr">
+      <c r="KW1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-04-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KT1" s="1" t="inlineStr">
+      <c r="KX1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-05-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KU1" s="1" t="inlineStr">
+      <c r="KY1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-06-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KV1" s="1" t="inlineStr">
+      <c r="KZ1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-07-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KW1" s="1" t="inlineStr">
+      <c r="LA1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-08-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KX1" s="1" t="inlineStr">
+      <c r="LB1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-09-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KY1" s="1" t="inlineStr">
+      <c r="LC1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-10-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="KZ1" s="1" t="inlineStr">
+      <c r="LD1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-11-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="LA1" s="1" t="inlineStr">
+      <c r="LE1" s="1" t="inlineStr">
         <is>
           <t>AOB 2023-12-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="LB1" s="1" t="inlineStr">
+      <c r="LF1" s="1" t="inlineStr">
         <is>
           <t>TOTAL_DMT_ACT</t>
         </is>
       </c>
-      <c r="LC1" s="1" t="inlineStr">
+      <c r="LG1" s="1" t="inlineStr">
         <is>
           <t>No. Reactivated DMT_ACT</t>
         </is>
       </c>
-      <c r="LD1" s="1" t="inlineStr">
+      <c r="LH1" s="1" t="inlineStr">
         <is>
           <t>DMT ACT 234 Cum No. Reactivated</t>
         </is>
       </c>
-      <c r="LE1" s="1" t="inlineStr">
+      <c r="LI1" s="1" t="inlineStr">
         <is>
           <t>% Reactivated DMT_ACT</t>
         </is>
       </c>
-      <c r="LF1" s="1" t="inlineStr">
+      <c r="LJ1" s="1" t="inlineStr">
         <is>
           <t>value_N'm</t>
         </is>
       </c>
-      <c r="LG1" s="1" t="inlineStr">
+      <c r="LK1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 318</t>
         </is>
       </c>
-      <c r="LH1" s="1" t="inlineStr">
+      <c r="LL1" s="1" t="inlineStr">
         <is>
           <t>POS ACTIVE</t>
         </is>
       </c>
-      <c r="LI1" s="1" t="inlineStr">
+      <c r="LM1" s="1" t="inlineStr">
         <is>
           <t>POS INACTIVE</t>
         </is>
       </c>
-      <c r="LJ1" s="1" t="inlineStr">
+      <c r="LN1" s="1" t="inlineStr">
         <is>
           <t>POS NEWLY DEPLOYED</t>
         </is>
       </c>
-      <c r="LK1" s="1" t="inlineStr">
+      <c r="LO1" s="1" t="inlineStr">
         <is>
           <t>POS RETRIEVED</t>
         </is>
       </c>
-      <c r="LL1" s="1" t="inlineStr">
+      <c r="LP1" s="1" t="inlineStr">
         <is>
           <t>VOLUME</t>
         </is>
       </c>
-      <c r="LM1" s="1" t="inlineStr">
+      <c r="LQ1" s="1" t="inlineStr">
         <is>
           <t>VALUE__2</t>
         </is>
       </c>
-      <c r="LN1" s="1" t="inlineStr">
+      <c r="LR1" s="1" t="inlineStr">
         <is>
           <t>COLL per ACTIVE POS</t>
         </is>
       </c>
-      <c r="LO1" s="1" t="inlineStr">
+      <c r="LS1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 326</t>
         </is>
       </c>
-      <c r="LP1" s="1" t="inlineStr">
+      <c r="LT1" s="1" t="inlineStr">
         <is>
           <t>NXP May-25</t>
         </is>
       </c>
-      <c r="LQ1" s="1" t="inlineStr">
+      <c r="LU1" s="1" t="inlineStr">
         <is>
           <t>NXP Jun-25</t>
         </is>
       </c>
-      <c r="LR1" s="1" t="inlineStr">
+      <c r="LV1" s="1" t="inlineStr">
         <is>
           <t>NXP Jul-25</t>
         </is>
       </c>
-      <c r="LS1" s="1" t="inlineStr">
+      <c r="LW1" s="1" t="inlineStr">
         <is>
           <t>NXP 2025 YTD VALUE</t>
         </is>
       </c>
-      <c r="LT1" s="1" t="inlineStr">
+      <c r="LX1" s="1" t="inlineStr">
         <is>
           <t>NXP 2025 YTD VALUE__2</t>
         </is>
       </c>
-      <c r="LU1" s="1" t="inlineStr">
+      <c r="LY1" s="1" t="inlineStr">
         <is>
           <t>NXP 2024 YTD VALUE</t>
         </is>
       </c>
-      <c r="LV1" s="1" t="inlineStr">
+      <c r="LZ1" s="1" t="inlineStr">
         <is>
           <t>NXP MOM VAR</t>
         </is>
       </c>
-      <c r="LW1" s="1" t="inlineStr">
+      <c r="MA1" s="1" t="inlineStr">
         <is>
           <t>NXP YOY VAR</t>
         </is>
       </c>
-      <c r="LX1" s="1" t="inlineStr">
+      <c r="MB1" s="1" t="inlineStr">
         <is>
           <t>NXP YTD BGT</t>
         </is>
       </c>
-      <c r="LY1" s="1" t="inlineStr">
+      <c r="MC1" s="1" t="inlineStr">
         <is>
           <t>NXP FULL YR BGT</t>
         </is>
       </c>
-      <c r="LZ1" s="1" t="inlineStr">
+      <c r="MD1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="MA1" s="1" t="inlineStr">
+      <c r="ME1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-02-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="MB1" s="1" t="inlineStr">
+      <c r="MF1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-03-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="MC1" s="1" t="inlineStr">
+      <c r="MG1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-04-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MD1" s="1" t="inlineStr">
+      <c r="MH1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-05-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="ME1" s="1" t="inlineStr">
+      <c r="MI1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-06-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MF1" s="1" t="inlineStr">
+      <c r="MJ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-07-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MG1" s="1" t="inlineStr">
+      <c r="MK1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-08-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MH1" s="1" t="inlineStr">
+      <c r="ML1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-09-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MI1" s="1" t="inlineStr">
+      <c r="MM1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-10-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MJ1" s="1" t="inlineStr">
+      <c r="MN1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-11-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MK1" s="1" t="inlineStr">
+      <c r="MO1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-12-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="ML1" s="1" t="inlineStr">
+      <c r="MP1" s="1" t="inlineStr">
         <is>
           <t>NXP RETAIL 2021-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="MM1" s="1" t="inlineStr">
+      <c r="MQ1" s="1" t="inlineStr">
         <is>
           <t>NXP 244 2021-02-01 00:00:00</t>
         </is>
       </c>
-      <c r="MN1" s="1" t="inlineStr">
+      <c r="MR1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-03-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MO1" s="1" t="inlineStr">
+      <c r="MS1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-04-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MP1" s="1" t="inlineStr">
+      <c r="MT1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-05-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MQ1" s="1" t="inlineStr">
+      <c r="MU1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-06-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MR1" s="1" t="inlineStr">
+      <c r="MV1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-07-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MS1" s="1" t="inlineStr">
+      <c r="MW1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-08-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MT1" s="1" t="inlineStr">
+      <c r="MX1" s="1" t="inlineStr">
         <is>
           <t>NXP 245 2021-09-01 00:00:00</t>
         </is>
       </c>
-      <c r="MU1" s="1" t="inlineStr">
+      <c r="MY1" s="1" t="inlineStr">
         <is>
           <t>NXP 246 2021-10-01 00:00:00</t>
         </is>
       </c>
-      <c r="MV1" s="1" t="inlineStr">
+      <c r="MZ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-11-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MW1" s="1" t="inlineStr">
+      <c r="NA1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-12-01 00:00:00__2</t>
         </is>
       </c>
-      <c r="MX1" s="1" t="inlineStr">
+      <c r="NB1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-01-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MY1" s="1" t="inlineStr">
+      <c r="NC1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-02-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="MZ1" s="1" t="inlineStr">
+      <c r="ND1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-03-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NA1" s="1" t="inlineStr">
+      <c r="NE1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-04-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NB1" s="1" t="inlineStr">
+      <c r="NF1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-05-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NC1" s="1" t="inlineStr">
+      <c r="NG1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-06-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="ND1" s="1" t="inlineStr">
+      <c r="NH1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-07-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NE1" s="1" t="inlineStr">
+      <c r="NI1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-08-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NF1" s="1" t="inlineStr">
+      <c r="NJ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-09-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NG1" s="1" t="inlineStr">
+      <c r="NK1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-10-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NH1" s="1" t="inlineStr">
+      <c r="NL1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-11-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NI1" s="1" t="inlineStr">
+      <c r="NM1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-12-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NJ1" s="1" t="inlineStr">
+      <c r="NN1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-01-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NK1" s="1" t="inlineStr">
+      <c r="NO1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-02-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NL1" s="1" t="inlineStr">
+      <c r="NP1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-03-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NM1" s="1" t="inlineStr">
+      <c r="NQ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-04-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NN1" s="1" t="inlineStr">
+      <c r="NR1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-05-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NO1" s="1" t="inlineStr">
+      <c r="NS1" s="1" t="inlineStr">
         <is>
           <t>CORPORATE</t>
         </is>
       </c>
-      <c r="NP1" s="1" t="inlineStr">
+      <c r="NT1" s="1" t="inlineStr">
         <is>
           <t>NXP CORPORATE 2020-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="NQ1" s="1" t="inlineStr">
+      <c r="NU1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-02-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NR1" s="1" t="inlineStr">
+      <c r="NV1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-03-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="NS1" s="1" t="inlineStr">
+      <c r="NW1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-04-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NT1" s="1" t="inlineStr">
+      <c r="NX1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-05-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NU1" s="1" t="inlineStr">
+      <c r="NY1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-06-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NV1" s="1" t="inlineStr">
+      <c r="NZ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-07-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NW1" s="1" t="inlineStr">
+      <c r="OA1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-08-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NX1" s="1" t="inlineStr">
+      <c r="OB1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-09-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NY1" s="1" t="inlineStr">
+      <c r="OC1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-10-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="NZ1" s="1" t="inlineStr">
+      <c r="OD1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-11-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OA1" s="1" t="inlineStr">
+      <c r="OE1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-12-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="OB1" s="1" t="inlineStr">
+      <c r="OF1" s="1" t="inlineStr">
         <is>
           <t>NXP CORPORATE 2021-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="OC1" s="1" t="inlineStr">
+      <c r="OG1" s="1" t="inlineStr">
         <is>
           <t>NXP 247 2021-02-01 00:00:00</t>
         </is>
       </c>
-      <c r="OD1" s="1" t="inlineStr">
+      <c r="OH1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-03-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OE1" s="1" t="inlineStr">
+      <c r="OI1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-04-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OF1" s="1" t="inlineStr">
+      <c r="OJ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-05-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OG1" s="1" t="inlineStr">
+      <c r="OK1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-06-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OH1" s="1" t="inlineStr">
+      <c r="OL1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-07-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OI1" s="1" t="inlineStr">
+      <c r="OM1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-08-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OJ1" s="1" t="inlineStr">
+      <c r="ON1" s="1" t="inlineStr">
         <is>
           <t>NXP 248 2021-09-01 00:00:00</t>
         </is>
       </c>
-      <c r="OK1" s="1" t="inlineStr">
+      <c r="OO1" s="1" t="inlineStr">
         <is>
           <t>NXP 249 2021-10-01 00:00:00</t>
         </is>
       </c>
-      <c r="OL1" s="1" t="inlineStr">
+      <c r="OP1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-11-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OM1" s="1" t="inlineStr">
+      <c r="OQ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-12-01 00:00:00__3</t>
         </is>
       </c>
-      <c r="ON1" s="1" t="inlineStr">
+      <c r="OR1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-01-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OO1" s="1" t="inlineStr">
+      <c r="OS1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-02-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OP1" s="1" t="inlineStr">
+      <c r="OT1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-03-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OQ1" s="1" t="inlineStr">
+      <c r="OU1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-04-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OR1" s="1" t="inlineStr">
+      <c r="OV1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-05-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OS1" s="1" t="inlineStr">
+      <c r="OW1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-06-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OT1" s="1" t="inlineStr">
+      <c r="OX1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-07-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OU1" s="1" t="inlineStr">
+      <c r="OY1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-08-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OV1" s="1" t="inlineStr">
+      <c r="OZ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-09-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OW1" s="1" t="inlineStr">
+      <c r="PA1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-10-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OX1" s="1" t="inlineStr">
+      <c r="PB1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-11-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OY1" s="1" t="inlineStr">
+      <c r="PC1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-12-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="OZ1" s="1" t="inlineStr">
+      <c r="PD1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-01-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PA1" s="1" t="inlineStr">
+      <c r="PE1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-02-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PB1" s="1" t="inlineStr">
+      <c r="PF1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-03-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PC1" s="1" t="inlineStr">
+      <c r="PG1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-04-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PD1" s="1" t="inlineStr">
+      <c r="PH1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-05-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PE1" s="1" t="inlineStr">
+      <c r="PI1" s="1" t="inlineStr">
         <is>
           <t>PUBLIC</t>
         </is>
       </c>
-      <c r="PF1" s="1" t="inlineStr">
+      <c r="PJ1" s="1" t="inlineStr">
         <is>
           <t>NXP PUBLIC 2020-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="PG1" s="1" t="inlineStr">
+      <c r="PK1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-02-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PH1" s="1" t="inlineStr">
+      <c r="PL1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-03-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PI1" s="1" t="inlineStr">
+      <c r="PM1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-04-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PJ1" s="1" t="inlineStr">
+      <c r="PN1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-05-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PK1" s="1" t="inlineStr">
+      <c r="PO1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-06-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PL1" s="1" t="inlineStr">
+      <c r="PP1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-07-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PM1" s="1" t="inlineStr">
+      <c r="PQ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-08-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PN1" s="1" t="inlineStr">
+      <c r="PR1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-09-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PO1" s="1" t="inlineStr">
+      <c r="PS1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-10-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PP1" s="1" t="inlineStr">
+      <c r="PT1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-11-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PQ1" s="1" t="inlineStr">
+      <c r="PU1" s="1" t="inlineStr">
         <is>
           <t>NXP 2020-12-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="PR1" s="1" t="inlineStr">
+      <c r="PV1" s="1" t="inlineStr">
         <is>
           <t>NXP PUBLIC 2021-01-01 00:00:00</t>
         </is>
       </c>
-      <c r="PS1" s="1" t="inlineStr">
+      <c r="PW1" s="1" t="inlineStr">
         <is>
           <t>NXP 250 2021-02-01 00:00:00</t>
         </is>
       </c>
-      <c r="PT1" s="1" t="inlineStr">
+      <c r="PX1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-03-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PU1" s="1" t="inlineStr">
+      <c r="PY1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-04-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PV1" s="1" t="inlineStr">
+      <c r="PZ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-05-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PW1" s="1" t="inlineStr">
+      <c r="QA1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-06-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PX1" s="1" t="inlineStr">
+      <c r="QB1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-07-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PY1" s="1" t="inlineStr">
+      <c r="QC1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-08-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="PZ1" s="1" t="inlineStr">
+      <c r="QD1" s="1" t="inlineStr">
         <is>
           <t>NXP 172 2021-09-01 00:00:00</t>
         </is>
       </c>
-      <c r="QA1" s="1" t="inlineStr">
+      <c r="QE1" s="1" t="inlineStr">
         <is>
           <t>NXP 173 2021-10-01 00:00:00</t>
         </is>
       </c>
-      <c r="QB1" s="1" t="inlineStr">
+      <c r="QF1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-11-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QC1" s="1" t="inlineStr">
+      <c r="QG1" s="1" t="inlineStr">
         <is>
           <t>NXP 2021-12-01 00:00:00__4</t>
         </is>
       </c>
-      <c r="QD1" s="1" t="inlineStr">
+      <c r="QH1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-01-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QE1" s="1" t="inlineStr">
+      <c r="QI1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-02-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QF1" s="1" t="inlineStr">
+      <c r="QJ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-03-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QG1" s="1" t="inlineStr">
+      <c r="QK1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-04-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QH1" s="1" t="inlineStr">
+      <c r="QL1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-05-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QI1" s="1" t="inlineStr">
+      <c r="QM1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-06-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QJ1" s="1" t="inlineStr">
+      <c r="QN1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-07-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QK1" s="1" t="inlineStr">
+      <c r="QO1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-08-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QL1" s="1" t="inlineStr">
+      <c r="QP1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-09-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QM1" s="1" t="inlineStr">
+      <c r="QQ1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-10-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QN1" s="1" t="inlineStr">
+      <c r="QR1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-11-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QO1" s="1" t="inlineStr">
+      <c r="QS1" s="1" t="inlineStr">
         <is>
           <t>NXP 2022-12-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QP1" s="1" t="inlineStr">
+      <c r="QT1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-01-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QQ1" s="1" t="inlineStr">
+      <c r="QU1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-02-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QR1" s="1" t="inlineStr">
+      <c r="QV1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-03-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QS1" s="1" t="inlineStr">
+      <c r="QW1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-04-01 00:00:00__5</t>
         </is>
       </c>
-      <c r="QT1" s="1" t="inlineStr">
+      <c r="QX1" s="1" t="inlineStr">
         <is>
           <t>NXP 2023-05-01 00:00:00__5</t>
         </is>

</xml_diff>

<commit_message>
Enhance narrative reporting: implement zero-case wording for various metrics, revert direct-upload review behavior, and add regression tests for coverage
</commit_message>
<xml_diff>
--- a/server/mpaStructure.xlsx
+++ b/server/mpaStructure.xlsx
@@ -506,49 +506,49 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>PBT 2018 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 15 2019 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 16 2020 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2021 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2022 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2023 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2024 YTD ACHVD</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>PBT 2025 YTD ACHVD__2</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>PBT 2025 YTD ACHVD</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 15 2019 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 16 2020 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2021 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2022 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2023 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2024 YTD ACHVD</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2025 YTD ACHVD__2</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>PBT 2026 YTD ACHVD</t>
-        </is>
-      </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PBT 2025 YOY VAR</t>
@@ -1761,17 +1761,17 @@
       </c>
       <c r="JG1" s="1" t="inlineStr">
         <is>
-          <t>CDS 1 CARDS MAY No. of Cards Issued</t>
+          <t>CDS1 No. of Cards Issued</t>
         </is>
       </c>
       <c r="JH1" s="1" t="inlineStr">
         <is>
-          <t>CDS 1 ACTIVE</t>
+          <t>CDS1 ACTIVE</t>
         </is>
       </c>
       <c r="JI1" s="1" t="inlineStr">
         <is>
-          <t>CDS 1 INACTIVE</t>
+          <t>CDS1 INACTIVE</t>
         </is>
       </c>
       <c r="JJ1" s="1" t="inlineStr">
@@ -1781,17 +1781,17 @@
       </c>
       <c r="JK1" s="1" t="inlineStr">
         <is>
-          <t>CDS 2 CARDS JUNE No. of Cards Issued</t>
+          <t>CDS2 No. of Cards Issued</t>
         </is>
       </c>
       <c r="JL1" s="1" t="inlineStr">
         <is>
-          <t>CDS 2 ACTIVE__2</t>
+          <t>CDS 2 ACTIVE</t>
         </is>
       </c>
       <c r="JM1" s="1" t="inlineStr">
         <is>
-          <t>CDS 2 INACTIVE__2</t>
+          <t>CDS2 INACTIVE</t>
         </is>
       </c>
       <c r="JN1" s="1" t="inlineStr">

</xml_diff>